<commit_message>
fix: 修复 A 列 No. 显示 1900/1/1 问题（Value+Style 同步覆盖）
</commit_message>
<xml_diff>
--- a/sample.xlsx
+++ b/sample.xlsx
@@ -153,7 +153,7 @@
       <patternFill/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -168,33 +168,50 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -525,66 +542,66 @@
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
+      <c r="E1" s="3"/>
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="3" t="s">
+      <c r="C2" s="3"/>
+      <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="3"/>
     </row>
     <row r="4" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="5"/>
+      <c r="E4" s="3"/>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
+      <c r="E5" s="3"/>
     </row>
     <row r="6" ht="172" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="3"/>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
@@ -593,7 +610,7 @@
       <c r="B7" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="5"/>
+      <c r="C7" s="3"/>
       <c r="D7" s="6" t="s">
         <v>15</v>
       </c>
@@ -605,14 +622,14 @@
       <c r="A8" s="7">
         <v>1</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="7" t="s">
+      <c r="C8" s="3"/>
+      <c r="D8" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="9">
         <v>46251</v>
       </c>
     </row>
@@ -620,14 +637,14 @@
       <c r="A9" s="7">
         <v>2</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="7" t="s">
+      <c r="C9" s="3"/>
+      <c r="D9" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="9">
         <v>46251</v>
       </c>
     </row>
@@ -635,14 +652,14 @@
       <c r="A10" s="7">
         <v>3</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="7" t="s">
+      <c r="C10" s="3"/>
+      <c r="D10" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="9">
         <v>46251</v>
       </c>
     </row>
@@ -650,29 +667,29 @@
       <c r="A11" s="7">
         <v>4</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="7" t="s">
+      <c r="C11" s="3"/>
+      <c r="D11" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="9">
         <v>46251</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="9">
+      <c r="A12" s="10">
         <v>5</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10" t="s">
+      <c r="C12" s="11"/>
+      <c r="D12" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="11">
+      <c r="E12" s="12">
         <v>46262</v>
       </c>
     </row>

</xml_diff>

<commit_message>
v0.9: rebuild template from 6-col human layout, all labels E col, values F col, A col numFmt pre-clean
</commit_message>
<xml_diff>
--- a/sample.xlsx
+++ b/sample.xlsx
@@ -14,27 +14,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>渠道部周例会会议纪要0817</t>
   </si>
   <si>
-    <t>时间(Time)</t>
+    <t>时间 (Time)</t>
   </si>
   <si>
     <t>2026年8月17日14:00-17:00</t>
   </si>
   <si>
-    <t>汇报人(Reporter)</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>参会人(Attendees)</t>
-  </si>
-  <si>
-    <t>赵伟富、潘勇超、朱世峰、张永建、李浩、潘燕、杭传龙、时永梅、王新娟、刘红宇、张军翔、盛哲泾、宋维叶、王雅文、高玉君、薛婧</t>
+    <t>地点 (Location)</t>
+  </si>
+  <si>
+    <t>汇报人 (Reporter)</t>
+  </si>
+  <si>
+    <t>参会人 (Attendees)</t>
+  </si>
+  <si>
+    <t>刘红宇、朱世峰</t>
   </si>
   <si>
     <t>请假人（Absentees）</t>
@@ -49,22 +49,7 @@
     <t>识野AI纪要</t>
   </si>
   <si>
-    <t>会议讨论内容要点及决议</t>
-  </si>
-  <si>
-    <t xml:space="preserve">一、Q3促销政策解读
-1、存储典配包下单门槛为 2 台起提，价格优于定制化备货；名额总量有限，实行先到先得。若约定期限内未提货，将取消统一存储定制资格，同时要求 8 月签单、8 月回款
-2、关注统一存储自主商机奖励，Q3新增的统一存储非指名商机奖励500元
-3、方案一体机下单编码未出，机卡分离出货，机头部分含返点，9月30号回款，整体数量有限
-4、G8 平台所有分销商须跟进签约事项；新平台政策预计本周发布，核心内容围绕两项：样机价格与促销包价格
-5、AI 软件已独立为单独部门，具备 AI 软件基础的分销商可关注并跟进相关政策；另据市场预测，5090dv2 涨价可能性较大，有需求的分销商请尽快报备锁定资源
-二、AI成果展示以及后续工作要求
-1、全体参会人员逐一汇报各自 AI 转型工作进展，围绕场景落地、能力建设、资源需求等内容展开交流，梳理现有成效与待解决问题，互通实践经验
-2、朱世峰数据还没上传还需要再完善模型；李浩预计下周完成模型的制作和对应的评估标准；张永建预计两周输出展示成果，搭建出初步模型
-3、各位同事已整理的数据须实现复用，地市及优选业务须依据看板数据推动后续工作落地；王雅文、高玉君须基于洞察识别出的高价值客户，切实推进业务转化与落地执行
-三、亿元达成情况
-1、梳理12 家亿元分销达成情况，武汉英信 1 亿档位尚未最终敲定，将结合分销商意愿跟进确认，部分分销商备货存在小幅风险需重点关注
-2、要求所有分销商 9 月上旬完成签约与备款筹备，提前规避后期项目、回款及划量不达标的风险</t>
+    <t>会议内容及决定</t>
   </si>
   <si>
     <t>No.</t>
@@ -79,31 +64,10 @@
     <t>完成时间</t>
   </si>
   <si>
-    <t>本次促销政策，方案一体机、6000D卡8月17日17:30分截止报备</t>
+    <t>测试</t>
   </si>
   <si>
     <t>片区经理</t>
-  </si>
-  <si>
-    <t>本周五片区经理将统一存储促销包推进情况反馈给刘红宇</t>
-  </si>
-  <si>
-    <t>片区经理/刘红宇</t>
-  </si>
-  <si>
-    <t>高玉君、王雅文、宋维叶、薛婧本周内讨论并输出客户洞察评估标准</t>
-  </si>
-  <si>
-    <t>高玉君、王雅文、宋维叶、薛婧</t>
-  </si>
-  <si>
-    <t>本周所有分销商完成G8平台签约，并完成G8促销政策宣贯</t>
-  </si>
-  <si>
-    <t>朱世峰、李浩下周完成AI模型的制作和对应的评估标准；张永建两周后交付初稿</t>
-  </si>
-  <si>
-    <t>朱世峰/李浩/张永建</t>
   </si>
 </sst>
 </file>
@@ -113,18 +77,13 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy/m/d"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <name val="微软雅黑"/>
     </font>
     <font>
       <b/>
@@ -145,15 +104,15 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC0C0C0"/>
-        <bgColor rgb="FFC0C0C0"/>
+        <fgColor rgb="00C0C0C0"/>
+        <bgColor rgb="00C0C0C0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -162,63 +121,38 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -525,188 +459,156 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="62" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="38" customWidth="1"/>
-    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="3" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="38" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
-      <c r="E1" s="3"/>
-    </row>
-    <row r="2" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="4" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="D2" s="3"/>
+      <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="3"/>
-    </row>
-    <row r="4" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="C3"/>
+      <c r="D3"/>
+      <c r="E3"/>
+      <c r="F3"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4"/>
+      <c r="D4"/>
+      <c r="E4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="F4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="3"/>
-    </row>
-    <row r="5" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
-      <c r="E5" s="3"/>
-    </row>
-    <row r="6" ht="172" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" ht="200" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="4"/>
+      <c r="B6"/>
+      <c r="C6"/>
+      <c r="D6"/>
+      <c r="E6"/>
+      <c r="F6"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="3"/>
-    </row>
-    <row r="7" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="B7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="6" t="s">
+      <c r="F7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="6" t="s">
+    </row>
+    <row r="8" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="5">
+        <v>1</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="7">
-        <v>1</v>
-      </c>
-      <c r="B8" s="5" t="s">
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="9">
+      <c r="F8" s="5">
         <v>46251</v>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="7">
-        <v>2</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E9" s="9">
-        <v>46251</v>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="7">
-        <v>3</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="E10" s="9">
-        <v>46251</v>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="7">
-        <v>4</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="3"/>
-      <c r="D11" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="E11" s="9">
-        <v>46251</v>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="10">
-        <v>5</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="E12" s="12">
-        <v>46262</v>
-      </c>
+    <row r="9" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="5"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+    </row>
+    <row r="10" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="5"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+    </row>
+    <row r="11" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="5"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
+  <mergeCells count="10">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B11:D11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>